<commit_message>
Add עומרי (Omri) as 6th employee — was missing from roster
6 employees now balance the schedule properly.
All constraints validated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shifts_29.3-4.4.xlsx
+++ b/shifts_29.3-4.4.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -90,32 +90,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FF00FF"/>
+        <bgColor rgb="00FF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6600"/>
+        <bgColor rgb="00FF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+        <bgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
         <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000B050"/>
-        <bgColor rgb="0000B050"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-        <bgColor rgb="00FF00FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000B0F0"/>
-        <bgColor rgb="0000B0F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -137,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,26 +157,32 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -618,37 +630,37 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
           <t>יהב</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>עומר</t>
+          <t>יהב</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>אורי</t>
+          <t>עומרי</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>משה</t>
         </is>
       </c>
     </row>
@@ -661,26 +673,26 @@
 14:00-22:00</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
@@ -688,12 +700,12 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>משה</t>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>עומרי</t>
         </is>
       </c>
     </row>
@@ -704,7 +716,7 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
@@ -716,32 +728,32 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>יהב</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>עומר</t>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>ניר</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>מקרא צבעים:</t>
         </is>
@@ -751,56 +763,66 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>יהב</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>סה״כ נקודות:</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>ניר: 5</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>משה: 5</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>עומר: 7</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>אורי: 5</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>יהב: 6</t>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>ניר: 6</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>משה: 4</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>עומר: 5</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>עומרי: 5</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>אורי: 4</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>יהב: 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enforce 5 weekly points before allowing 6 (tiered scheduling)
Tier 1: assign employees under their target (5 pts, or custom override)
Tier 2: allow target+1 (6 pts) only when no one is under target
Tier 3: fallback ignoring points (last resort)

Sorting by weekly points first ensures everyone hits 5 before
anyone gets a 6th point.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shifts_29.3-4.4.xlsx
+++ b/shifts_29.3-4.4.xlsx
@@ -90,38 +90,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6600"/>
+        <bgColor rgb="00FF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FF00FF"/>
         <bgColor rgb="00FF00FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF6600"/>
-        <bgColor rgb="00FF6600"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0000B050"/>
         <bgColor rgb="0000B050"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000B0F0"/>
-        <bgColor rgb="0000B0F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,10 +157,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,20 +169,20 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -630,35 +630,35 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>משה</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -675,37 +675,37 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>עומרי</t>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>אורי</t>
         </is>
       </c>
     </row>
@@ -716,37 +716,37 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -758,7 +758,7 @@
           <t>מקרא צבעים:</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -768,7 +768,7 @@
           <t>משה</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
@@ -778,7 +778,7 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
@@ -812,17 +812,17 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>עומרי: 5</t>
+          <t>עומרי: 6</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>אורי: 4</t>
+          <t>אורי: 5</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>יהב: 4</t>
+          <t>יהב: 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Smart urgency-based scheduling: ensures everyone reaches 5 points
- Calculate remaining available slots per employee per week
- Prioritize employees with fewer opportunities to reach target
- Yahav: target 1 shift/week (allow 2 if needed)
- Fixes issue where constrained employees ended below target

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shifts_29.3-4.4.xlsx
+++ b/shifts_29.3-4.4.xlsx
@@ -90,38 +90,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FF00FF"/>
+        <bgColor rgb="00FF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
         <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B0F0"/>
-        <bgColor rgb="0000B0F0"/>
+        <fgColor rgb="0000B050"/>
+        <bgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FF6600"/>
         <bgColor rgb="00FF6600"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-        <bgColor rgb="00FF00FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0000B050"/>
-        <bgColor rgb="0000B050"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,32 +157,32 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -630,37 +630,37 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
         </is>
       </c>
     </row>
@@ -673,39 +673,39 @@
 14:00-22:00</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>יהב</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>ניר</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>אורי</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>אורי</t>
         </is>
       </c>
     </row>
@@ -716,39 +716,39 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>אורי</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>עומרי</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>ניר</t>
+          <t>יהב</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>אורי</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
           <t>משה</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
@@ -778,7 +778,7 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>אורי</t>
         </is>
@@ -797,12 +797,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 6</t>
+          <t>ניר: 5</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 4</t>
+          <t>משה: 5</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>עומרי: 6</t>
+          <t>עומרי: 5</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>אורי: 5</t>
+          <t>אורי: 6</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">

</xml_diff>